<commit_message>
agentic-qe-mvp: Flow 2 is hotel booking release 2.0 (AQPI-32 + demo/hotel-booking-platform-v2) on the hotel baseline; commission engine removed from the demo; Test Lab uses hotel rules
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
@@ -161,7 +161,7 @@
     <t>sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef)</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T04:13:45.754Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T15:08:27.184Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -1377,7 +1377,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T04:13:46.483Z</t>
+    <t>2026-10-02T15:08:28.180Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -1518,7 +1518,7 @@
     <t>End-to-end testing from the user's point of view</t>
   </si>
   <si>
-    <t>Steers the design agents to write browser journeys as the travel advisor experiences them.</t>
+    <t>Steers the design agents to write journeys as the guest experiences them, from search to confirmation.</t>
   </si>
   <si>
     <t>testcases, scripts, execution</t>
@@ -5548,7 +5548,7 @@
         <v>387</v>
       </c>
       <c r="E2" s="2">
-        <v>1028</v>
+        <v>1115</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -5566,7 +5566,7 @@
         <v>387</v>
       </c>
       <c r="E3" s="2">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -5584,7 +5584,7 @@
         <v>387</v>
       </c>
       <c r="E4" s="2">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -5602,7 +5602,7 @@
         <v>387</v>
       </c>
       <c r="E5" s="2">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -5620,7 +5620,7 @@
         <v>387</v>
       </c>
       <c r="E6" s="2">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -5638,7 +5638,7 @@
         <v>387</v>
       </c>
       <c r="E7" s="2">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -5656,7 +5656,7 @@
         <v>387</v>
       </c>
       <c r="E8" s="2">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -5674,7 +5674,7 @@
         <v>387</v>
       </c>
       <c r="E9" s="2">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="F9" s="2"/>
     </row>

</xml_diff>

<commit_message>
agentic-qe-mvp: QE lead report lists each input's stories (AQPI-33 to AQPI-36 for release 2.0)
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
@@ -161,7 +161,7 @@
     <t>sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef)</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T15:08:27.184Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T15:29:42.911Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -1377,7 +1377,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T15:08:28.180Z</t>
+    <t>2026-10-02T15:29:43.709Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -5548,7 +5548,7 @@
         <v>387</v>
       </c>
       <c r="E2" s="2">
-        <v>1115</v>
+        <v>1142</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -5566,7 +5566,7 @@
         <v>387</v>
       </c>
       <c r="E3" s="2">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -5584,7 +5584,7 @@
         <v>387</v>
       </c>
       <c r="E4" s="2">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -5602,7 +5602,7 @@
         <v>387</v>
       </c>
       <c r="E5" s="2">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -5620,7 +5620,7 @@
         <v>387</v>
       </c>
       <c r="E6" s="2">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -5638,7 +5638,7 @@
         <v>387</v>
       </c>
       <c r="E7" s="2">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -5656,7 +5656,7 @@
         <v>387</v>
       </c>
       <c r="E8" s="2">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -5674,7 +5674,7 @@
         <v>387</v>
       </c>
       <c r="E9" s="2">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F9" s="2"/>
     </row>

</xml_diff>

<commit_message>
agentic-qe-mvp: traceability matrix, Jira defects linked to their story, enterprise skill upload
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
@@ -12,16 +12,18 @@
     <sheet sheetId="6" name="Defects" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Coverage" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Attribute coverage" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Approvals" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Skills" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="Hand-overs" state="visible" r:id="rId14"/>
+    <sheet sheetId="9" name="Traceability by story" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Traceability matrix" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Approvals" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Skills" state="visible" r:id="rId15"/>
+    <sheet sheetId="13" name="Hand-overs" state="visible" r:id="rId16"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1324" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="638">
   <si>
     <t>Metric</t>
   </si>
@@ -167,7 +169,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T16:18:27.590Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (35af1ef) at 2026-10-02T19:27:46.786Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -1218,6 +1220,12 @@
     <t>Severity</t>
   </si>
   <si>
+    <t>Story</t>
+  </si>
+  <si>
+    <t>Jira defect</t>
+  </si>
+  <si>
     <t>Expected</t>
   </si>
   <si>
@@ -1359,6 +1367,303 @@
     <t>Prefix of the Idempotency-Key sent with a reservation (the full key is 8 to 64 characters)</t>
   </si>
   <si>
+    <t>Jira item</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Parent</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>initiative</t>
+  </si>
+  <si>
+    <t>[Initiative] Intelligent Hotel Shopping and Reservation Experience</t>
+  </si>
+  <si>
+    <t>verified</t>
+  </si>
+  <si>
+    <t>AQPI-2</t>
+  </si>
+  <si>
+    <t>epic</t>
+  </si>
+  <si>
+    <t>[Epic 1] Search and Availability</t>
+  </si>
+  <si>
+    <t>AQPI-3</t>
+  </si>
+  <si>
+    <t>story</t>
+  </si>
+  <si>
+    <t>3.1 Search hotels by destination and date range</t>
+  </si>
+  <si>
+    <t>AQPI-4</t>
+  </si>
+  <si>
+    <t>3.2 Validate occupancy and stay criteria</t>
+  </si>
+  <si>
+    <t>AQPI-5</t>
+  </si>
+  <si>
+    <t>3.3 Handle unavailable or failed searches</t>
+  </si>
+  <si>
+    <t>AQPI-6</t>
+  </si>
+  <si>
+    <t>[Epic 2] Hotel Results and Selection</t>
+  </si>
+  <si>
+    <t>AQPI-7</t>
+  </si>
+  <si>
+    <t>4.1 Display available hotels</t>
+  </si>
+  <si>
+    <t>AQPI-8</t>
+  </si>
+  <si>
+    <t>4.2 Sort and filter hotel results</t>
+  </si>
+  <si>
+    <t>AQPI-9</t>
+  </si>
+  <si>
+    <t>4.3 View hotel and room details</t>
+  </si>
+  <si>
+    <t>AQPI-10</t>
+  </si>
+  <si>
+    <t>[Epic 3] Personalized Ancillary Offers</t>
+  </si>
+  <si>
+    <t>AQPI-11</t>
+  </si>
+  <si>
+    <t>5.1 Determine eligible ancillary offers</t>
+  </si>
+  <si>
+    <t>AQPI-12</t>
+  </si>
+  <si>
+    <t>5.2 Display ancillary offers</t>
+  </si>
+  <si>
+    <t>AQPI-13</t>
+  </si>
+  <si>
+    <t>5.3 Explain and control personalization</t>
+  </si>
+  <si>
+    <t>AQPI-14</t>
+  </si>
+  <si>
+    <t>[Epic 4] Cart Management</t>
+  </si>
+  <si>
+    <t>AQPI-15</t>
+  </si>
+  <si>
+    <t>6.1 Add room selection to cart</t>
+  </si>
+  <si>
+    <t>AQPI-16</t>
+  </si>
+  <si>
+    <t>6.2 Add, update, and remove ancillaries</t>
+  </si>
+  <si>
+    <t>AQPI-17</t>
+  </si>
+  <si>
+    <t>6.3 Review cart and total price</t>
+  </si>
+  <si>
+    <t>AQPI-18</t>
+  </si>
+  <si>
+    <t>[Epic 5] Checkout and Reservation</t>
+  </si>
+  <si>
+    <t>AQPI-19</t>
+  </si>
+  <si>
+    <t>7.1 Capture guest and contact information</t>
+  </si>
+  <si>
+    <t>AQPI-20</t>
+  </si>
+  <si>
+    <t>7.2 Capture and authorize payment</t>
+  </si>
+  <si>
+    <t>AQPI-21</t>
+  </si>
+  <si>
+    <t>7.3 Create reservation idempotently</t>
+  </si>
+  <si>
+    <t>AQPI-22</t>
+  </si>
+  <si>
+    <t>7.4 Show booking outcome</t>
+  </si>
+  <si>
+    <t>AQPI-23</t>
+  </si>
+  <si>
+    <t>[Epic 6] Confirmation and Notifications</t>
+  </si>
+  <si>
+    <t>AQPI-24</t>
+  </si>
+  <si>
+    <t>8.1 Generate confirmation message</t>
+  </si>
+  <si>
+    <t>AQPI-25</t>
+  </si>
+  <si>
+    <t>8.2 Send and track confirmation email</t>
+  </si>
+  <si>
+    <t>AQPI-26</t>
+  </si>
+  <si>
+    <t>8.3 Resend confirmation safely</t>
+  </si>
+  <si>
+    <t>AQPI-27</t>
+  </si>
+  <si>
+    <t>[Epic 7] Cross-Cutting Quality, Privacy and Observability</t>
+  </si>
+  <si>
+    <t>AQPI-28</t>
+  </si>
+  <si>
+    <t>9.1 Protect sensitive data</t>
+  </si>
+  <si>
+    <t>AQPI-29</t>
+  </si>
+  <si>
+    <t>9.2 Provide end-to-end observability</t>
+  </si>
+  <si>
+    <t>AQPI-30</t>
+  </si>
+  <si>
+    <t>9.3 Meet accessibility requirements</t>
+  </si>
+  <si>
+    <t>AQPI-31</t>
+  </si>
+  <si>
+    <t>9.4 Meet performance and reliability objectives</t>
+  </si>
+  <si>
+    <t>Jira</t>
+  </si>
+  <si>
+    <t>Requirement text</t>
+  </si>
+  <si>
+    <t>Rule</t>
+  </si>
+  <si>
+    <t>Test case</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>Test data</t>
+  </si>
+  <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>Defect</t>
+  </si>
+  <si>
+    <t>BR-001</t>
+  </si>
+  <si>
+    <t>TD-F-001</t>
+  </si>
+  <si>
+    <t>br-001-booking-journey.spec.js</t>
+  </si>
+  <si>
+    <t>TD-F-002</t>
+  </si>
+  <si>
+    <t>BR-002</t>
+  </si>
+  <si>
+    <t>TD-F-003</t>
+  </si>
+  <si>
+    <t>br-002-bookable-inventory.spec.js</t>
+  </si>
+  <si>
+    <t>BR-004</t>
+  </si>
+  <si>
+    <t>TD-F-004</t>
+  </si>
+  <si>
+    <t>br-004-offers-not-blocking.spec.js</t>
+  </si>
+  <si>
+    <t>BR-005</t>
+  </si>
+  <si>
+    <t>TD-F-005</t>
+  </si>
+  <si>
+    <t>br-005-duplicate-submission.spec.js</t>
+  </si>
+  <si>
+    <t>BR-006</t>
+  </si>
+  <si>
+    <t>TD-F-006</t>
+  </si>
+  <si>
+    <t>br-006-durable-confirmation.spec.js</t>
+  </si>
+  <si>
+    <t>BR-007</t>
+  </si>
+  <si>
+    <t>TD-F-007</t>
+  </si>
+  <si>
+    <t>br-007-confirmation-shown.spec.js</t>
+  </si>
+  <si>
+    <t>BR-051</t>
+  </si>
+  <si>
+    <t>TD-F-008</t>
+  </si>
+  <si>
+    <t>br-051-offers-not-blocking.spec.js</t>
+  </si>
+  <si>
     <t>Gate</t>
   </si>
   <si>
@@ -1383,7 +1688,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T16:18:28.425Z</t>
+    <t>2026-10-02T19:27:47.566Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -2223,6 +2528,451 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="50" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="9" width="11" customWidth="1"/>
+    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>512</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>535</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>339</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>545</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>547</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>549</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2235,189 +2985,189 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>449</v>
+        <v>550</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>314</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>450</v>
+        <v>551</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>451</v>
+        <v>552</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>452</v>
+        <v>553</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>453</v>
+        <v>554</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>454</v>
+        <v>555</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>455</v>
+        <v>556</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>456</v>
+        <v>557</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>457</v>
+        <v>558</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>458</v>
+        <v>559</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>459</v>
+        <v>560</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>460</v>
+        <v>561</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>461</v>
+        <v>562</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>462</v>
+        <v>563</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>463</v>
+        <v>564</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>464</v>
+        <v>565</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>465</v>
+        <v>566</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>466</v>
+        <v>567</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>467</v>
+        <v>568</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>468</v>
+        <v>569</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>469</v>
+        <v>570</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>470</v>
+        <v>571</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>471</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>472</v>
+        <v>573</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>473</v>
+        <v>574</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>474</v>
+        <v>575</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>475</v>
+        <v>576</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>476</v>
+        <v>577</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>477</v>
+        <v>578</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>478</v>
+        <v>579</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>479</v>
+        <v>580</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>480</v>
+        <v>581</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>481</v>
+        <v>582</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>482</v>
+        <v>583</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>483</v>
+        <v>584</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>484</v>
+        <v>585</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>485</v>
+        <v>586</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>486</v>
+        <v>587</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>487</v>
+        <v>588</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>488</v>
+        <v>589</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>489</v>
+        <v>590</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>490</v>
+        <v>591</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>491</v>
+        <v>592</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>492</v>
+        <v>593</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>493</v>
+        <v>594</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>494</v>
+        <v>595</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>495</v>
+        <v>596</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>496</v>
+        <v>597</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>497</v>
+        <v>598</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>498</v>
+        <v>599</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>499</v>
+        <v>600</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>500</v>
+        <v>601</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>501</v>
+        <v>602</v>
       </c>
     </row>
   </sheetData>
@@ -2426,7 +3176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2440,186 +3190,186 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>502</v>
+        <v>603</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>503</v>
+        <v>604</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>504</v>
+        <v>605</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>505</v>
+        <v>606</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>506</v>
+        <v>607</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>507</v>
+        <v>608</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>508</v>
+        <v>609</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>510</v>
+        <v>611</v>
       </c>
     </row>
     <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>477</v>
+        <v>578</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>511</v>
+        <v>612</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>512</v>
+        <v>613</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>497</v>
+        <v>598</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>513</v>
+        <v>614</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>514</v>
+        <v>615</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>515</v>
+        <v>616</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>516</v>
+        <v>617</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>517</v>
+        <v>618</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>518</v>
+        <v>619</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>519</v>
+        <v>620</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>520</v>
+        <v>621</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>521</v>
+        <v>622</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>522</v>
+        <v>623</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>523</v>
+        <v>624</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>524</v>
+        <v>625</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>525</v>
+        <v>626</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>526</v>
+        <v>627</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>527</v>
+        <v>628</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>528</v>
+        <v>629</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>529</v>
+        <v>630</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>530</v>
+        <v>631</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>531</v>
+        <v>632</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>532</v>
+        <v>633</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>533</v>
+        <v>634</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>534</v>
+        <v>635</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>535</v>
+        <v>636</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>509</v>
+        <v>610</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>536</v>
+        <v>637</v>
       </c>
     </row>
   </sheetData>
@@ -5554,7 +6304,7 @@
         <v>389</v>
       </c>
       <c r="E2" s="2">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -5572,7 +6322,7 @@
         <v>389</v>
       </c>
       <c r="E3" s="2">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -5590,7 +6340,7 @@
         <v>389</v>
       </c>
       <c r="E4" s="2">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -5608,7 +6358,7 @@
         <v>389</v>
       </c>
       <c r="E5" s="2">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -5626,7 +6376,7 @@
         <v>389</v>
       </c>
       <c r="E6" s="2">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -5644,7 +6394,7 @@
         <v>389</v>
       </c>
       <c r="E7" s="2">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -5662,7 +6412,7 @@
         <v>389</v>
       </c>
       <c r="E8" s="2">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -5692,18 +6442,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="8" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
+    <col min="11" max="11" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
@@ -5714,22 +6466,28 @@
         <v>391</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>393</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>394</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>395</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -5756,16 +6514,16 @@
         <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>337</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>23</v>
@@ -5794,7 +6552,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5817,7 +6575,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5840,7 +6598,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5863,7 +6621,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5886,7 +6644,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5909,7 +6667,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5932,7 +6690,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5955,7 +6713,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -5978,7 +6736,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6001,7 +6759,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6024,7 +6782,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6047,7 +6805,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6070,7 +6828,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6093,7 +6851,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6116,7 +6874,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6139,7 +6897,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6162,7 +6920,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6185,7 +6943,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6208,7 +6966,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6231,7 +6989,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6254,7 +7012,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6277,7 +7035,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6300,7 +7058,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6323,7 +7081,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6346,7 +7104,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6369,7 +7127,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6392,7 +7150,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6415,7 +7173,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6438,7 +7196,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6461,7 +7219,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6484,7 +7242,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6507,7 +7265,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6530,7 +7288,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6553,7 +7311,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6576,7 +7334,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6599,7 +7357,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6622,7 +7380,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6645,7 +7403,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6668,7 +7426,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6691,7 +7449,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6714,7 +7472,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6737,7 +7495,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6760,7 +7518,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6783,7 +7541,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6806,7 +7564,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6829,7 +7587,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6852,7 +7610,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="49" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6875,7 +7633,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="50" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6898,7 +7656,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="51" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6921,7 +7679,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6944,7 +7702,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6967,7 +7725,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -6990,7 +7748,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7013,7 +7771,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7036,7 +7794,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7059,7 +7817,7 @@
         <v>0</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7082,7 +7840,7 @@
         <v>0</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7105,7 +7863,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="60" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7128,7 +7886,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7151,7 +7909,7 @@
         <v>0</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7174,7 +7932,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7197,7 +7955,7 @@
         <v>0</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7220,7 +7978,7 @@
         <v>0</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="65" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7243,7 +8001,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="66" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7266,7 +8024,7 @@
         <v>0</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7289,7 +8047,7 @@
         <v>0</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="68" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7312,7 +8070,7 @@
         <v>0</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="69" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7335,7 +8093,7 @@
         <v>0</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="70" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7358,7 +8116,7 @@
         <v>0</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="71" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7381,7 +8139,7 @@
         <v>0</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="72" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7404,7 +8162,7 @@
         <v>0</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="73" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7427,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="74" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7450,7 +8208,7 @@
         <v>0</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="75" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7473,7 +8231,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="76" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7496,7 +8254,7 @@
         <v>0</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="77" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7519,7 +8277,7 @@
         <v>0</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="78" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7542,7 +8300,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="79" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7565,7 +8323,7 @@
         <v>0</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="80" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7588,7 +8346,7 @@
         <v>0</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="81" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7611,7 +8369,7 @@
         <v>0</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="82" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7634,7 +8392,7 @@
         <v>0</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="83" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7657,7 +8415,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="84" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7680,7 +8438,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="85" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7703,7 +8461,7 @@
         <v>0</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="86" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7726,7 +8484,7 @@
         <v>0</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="87" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7749,7 +8507,7 @@
         <v>0</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="88" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7772,7 +8530,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="89" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7795,7 +8553,7 @@
         <v>0</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="90" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7818,7 +8576,7 @@
         <v>0</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="91" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7841,7 +8599,7 @@
         <v>0</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="92" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7864,7 +8622,7 @@
         <v>0</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="93" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7887,7 +8645,7 @@
         <v>0</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="94" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7910,7 +8668,7 @@
         <v>0</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="95" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7933,7 +8691,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="96" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7956,7 +8714,7 @@
         <v>0</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="97" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -7979,7 +8737,7 @@
         <v>0</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="98" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8002,7 +8760,7 @@
         <v>0</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="99" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8025,7 +8783,7 @@
         <v>0</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="100" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8048,7 +8806,7 @@
         <v>0</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="101" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8071,7 +8829,7 @@
         <v>0</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="102" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8094,7 +8852,7 @@
         <v>0</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="103" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8117,7 +8875,7 @@
         <v>0</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="104" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8140,7 +8898,7 @@
         <v>0</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="105" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8163,7 +8921,7 @@
         <v>0</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="106" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8186,7 +8944,7 @@
         <v>0</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="107" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8209,7 +8967,7 @@
         <v>0</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="108" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8232,7 +8990,7 @@
         <v>0</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="109" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8255,7 +9013,7 @@
         <v>0</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="110" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8278,7 +9036,7 @@
         <v>0</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8301,7 +9059,7 @@
         <v>0</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="112" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8324,7 +9082,7 @@
         <v>0</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="113" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8347,7 +9105,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="114" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8370,7 +9128,7 @@
         <v>0</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="115" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8393,7 +9151,7 @@
         <v>0</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="116" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8416,7 +9174,7 @@
         <v>0</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="117" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8439,7 +9197,7 @@
         <v>0</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="118" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8462,7 +9220,7 @@
         <v>0</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="119" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8485,7 +9243,7 @@
         <v>0</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="120" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8508,7 +9266,7 @@
         <v>0</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="121" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8531,7 +9289,7 @@
         <v>0</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="122" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8554,7 +9312,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="123" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8577,7 +9335,7 @@
         <v>0</v>
       </c>
       <c r="G123" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="124" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8600,7 +9358,7 @@
         <v>0</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="125" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8623,7 +9381,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="126" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8646,7 +9404,7 @@
         <v>0</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="127" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8669,7 +9427,7 @@
         <v>0</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="128" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8692,7 +9450,7 @@
         <v>0</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="129" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -8715,7 +9473,7 @@
         <v>0</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -8737,13 +9495,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
@@ -8751,212 +9509,212 @@
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>340</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="13" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>339</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="16" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>362</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
   </sheetData>
@@ -8967,48 +9725,1136 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="80" customWidth="1"/>
+    <col min="1" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="10" customWidth="1"/>
+    <col min="8" max="9" width="8" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>444</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>445</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>446</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2">
+        <v>6</v>
+      </c>
+      <c r="F2" s="2">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>447</v>
       </c>
-      <c r="E2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>448</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="E16" s="2">
+        <v>0</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="E17" s="2">
+        <v>0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="E21" s="2">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="E22" s="2">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="E23" s="2">
+        <v>0</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2">
+        <v>0</v>
+      </c>
+      <c r="I23" s="2">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="E24" s="2">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E29" s="2">
+        <v>0</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E30" s="2">
+        <v>0</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="E31" s="2">
+        <v>0</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="E32" s="2">
+        <v>0</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Traceability: an incremental cycle's 'By Jira item' view and Excel sheet include the baseline stories it re-tested (scope column); defects prefer this cycle's stories
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="641">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1681" uniqueCount="643">
   <si>
     <t>Metric</t>
   </si>
@@ -170,7 +170,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) at 2026-10-02T20:05:08.555Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) at 2026-10-02T20:26:12.623Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -1383,6 +1383,9 @@
     <t>Level</t>
   </si>
   <si>
+    <t>Scope</t>
+  </si>
+  <si>
     <t>Parent</t>
   </si>
   <si>
@@ -1392,6 +1395,9 @@
     <t>initiative</t>
   </si>
   <si>
+    <t>this cycle</t>
+  </si>
+  <si>
     <t>[Initiative] Intelligent Hotel Shopping and Reservation Experience</t>
   </si>
   <si>
@@ -1698,7 +1704,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T20:05:09.333Z</t>
+    <t>2026-10-02T20:26:13.414Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -2538,19 +2544,19 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="8" max="9" width="8" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="1" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="10" customWidth="1"/>
+    <col min="9" max="10" width="8" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>444</v>
       </c>
@@ -2564,45 +2570,48 @@
         <v>447</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="E2" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="F2" s="2">
         <v>6</v>
-      </c>
-      <c r="F2" s="2">
-        <v>7</v>
       </c>
       <c r="G2" s="2">
         <v>7</v>
@@ -2611,1062 +2620,1155 @@
         <v>7</v>
       </c>
       <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>0</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2">
+        <v>0</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>0</v>
+      </c>
+      <c r="H5" s="2">
+        <v>0</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>453</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0</v>
+      </c>
+      <c r="H6" s="2">
+        <v>0</v>
+      </c>
+      <c r="I6" s="2">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0</v>
+      </c>
+      <c r="H7" s="2">
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0</v>
+      </c>
+      <c r="H8" s="2">
+        <v>0</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0</v>
+      </c>
+      <c r="H9" s="2">
+        <v>0</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>463</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2">
+        <v>0</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F13" s="2">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="H14" s="2">
+        <v>0</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0</v>
+      </c>
+      <c r="J14" s="2">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="E3" s="2">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2">
-        <v>0</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>480</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>0</v>
+      </c>
+      <c r="H15" s="2">
+        <v>0</v>
+      </c>
+      <c r="I15" s="2">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <v>0</v>
+      </c>
+      <c r="K15" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="L15" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F16" s="2">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0</v>
+      </c>
+      <c r="H16" s="2">
+        <v>0</v>
+      </c>
+      <c r="I16" s="2">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2">
+        <v>0</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="F17" s="2">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0</v>
+      </c>
+      <c r="H17" s="2">
+        <v>0</v>
+      </c>
+      <c r="I17" s="2">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2">
+        <v>0</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0</v>
+      </c>
+      <c r="H18" s="2">
+        <v>0</v>
+      </c>
+      <c r="I18" s="2">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2">
+        <v>0</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>454</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>456</v>
-      </c>
-      <c r="E4" s="2">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2">
-        <v>0</v>
-      </c>
-      <c r="I4" s="2">
-        <v>0</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="C19" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0</v>
+      </c>
+      <c r="H19" s="2">
+        <v>0</v>
+      </c>
+      <c r="I19" s="2">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2">
+        <v>0</v>
+      </c>
+      <c r="K19" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="L19" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2">
-        <v>0</v>
-      </c>
-      <c r="G5" s="2">
-        <v>0</v>
-      </c>
-      <c r="H5" s="2">
-        <v>0</v>
-      </c>
-      <c r="I5" s="2">
-        <v>0</v>
-      </c>
-      <c r="J5" s="2" t="s">
+      <c r="C20" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>459</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>451</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2">
-        <v>0</v>
-      </c>
-      <c r="I6" s="2">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="L20" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0</v>
+      </c>
+      <c r="K21" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="L21" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="F22" s="2">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2">
+        <v>0</v>
+      </c>
+      <c r="H22" s="2">
+        <v>0</v>
+      </c>
+      <c r="I22" s="2">
+        <v>0</v>
+      </c>
+      <c r="J22" s="2">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="F23" s="2">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2">
+        <v>0</v>
+      </c>
+      <c r="H23" s="2">
+        <v>0</v>
+      </c>
+      <c r="I23" s="2">
+        <v>0</v>
+      </c>
+      <c r="J23" s="2">
+        <v>0</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
-        <v>0</v>
-      </c>
-      <c r="H7" s="2">
-        <v>0</v>
-      </c>
-      <c r="I7" s="2">
-        <v>0</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="E24" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="F24" s="2">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2">
-        <v>0</v>
-      </c>
-      <c r="H8" s="2">
-        <v>0</v>
-      </c>
-      <c r="I8" s="2">
-        <v>0</v>
-      </c>
-      <c r="J8" s="2" t="s">
+      <c r="L24" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="G9" s="2">
-        <v>0</v>
-      </c>
-      <c r="H9" s="2">
-        <v>0</v>
-      </c>
-      <c r="I9" s="2">
-        <v>0</v>
-      </c>
-      <c r="J9" s="2" t="s">
+      <c r="L25" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>467</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>461</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2" t="s">
+      <c r="L26" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0</v>
+      </c>
+      <c r="G27" s="2">
+        <v>0</v>
+      </c>
+      <c r="H27" s="2">
+        <v>0</v>
+      </c>
+      <c r="I27" s="2">
+        <v>0</v>
+      </c>
+      <c r="J27" s="2">
+        <v>0</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="L27" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0</v>
-      </c>
-      <c r="F11" s="2">
-        <v>0</v>
-      </c>
-      <c r="G11" s="2">
-        <v>0</v>
-      </c>
-      <c r="H11" s="2">
-        <v>0</v>
-      </c>
-      <c r="I11" s="2">
-        <v>0</v>
-      </c>
-      <c r="J11" s="2" t="s">
+      <c r="E28" s="2" t="s">
+        <v>506</v>
+      </c>
+      <c r="F28" s="2">
+        <v>0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>0</v>
+      </c>
+      <c r="H28" s="2">
+        <v>0</v>
+      </c>
+      <c r="I28" s="2">
+        <v>0</v>
+      </c>
+      <c r="J28" s="2">
+        <v>0</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="E12" s="2">
-        <v>0</v>
-      </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2">
-        <v>0</v>
-      </c>
-      <c r="H12" s="2">
-        <v>0</v>
-      </c>
-      <c r="I12" s="2">
-        <v>0</v>
-      </c>
-      <c r="J12" s="2" t="s">
+      <c r="L28" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="F29" s="2">
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <v>0</v>
+      </c>
+      <c r="I29" s="2">
+        <v>0</v>
+      </c>
+      <c r="J29" s="2">
+        <v>0</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="E13" s="2">
-        <v>1</v>
-      </c>
-      <c r="F13" s="2">
-        <v>1</v>
-      </c>
-      <c r="G13" s="2">
-        <v>1</v>
-      </c>
-      <c r="H13" s="2">
-        <v>1</v>
-      </c>
-      <c r="I13" s="2">
-        <v>0</v>
-      </c>
-      <c r="J13" s="2" t="s">
+      <c r="L29" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="F30" s="2">
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <v>0</v>
+      </c>
+      <c r="I30" s="2">
+        <v>0</v>
+      </c>
+      <c r="J30" s="2">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L30" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>476</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2">
-        <v>0</v>
-      </c>
-      <c r="I14" s="2">
-        <v>0</v>
-      </c>
-      <c r="J14" s="2" t="s">
+      <c r="D31" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>512</v>
+      </c>
+      <c r="F31" s="2">
+        <v>0</v>
+      </c>
+      <c r="G31" s="2">
+        <v>0</v>
+      </c>
+      <c r="H31" s="2">
+        <v>0</v>
+      </c>
+      <c r="I31" s="2">
+        <v>0</v>
+      </c>
+      <c r="J31" s="2">
+        <v>0</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="E15" s="2">
-        <v>0</v>
-      </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2">
-        <v>0</v>
-      </c>
-      <c r="H15" s="2">
-        <v>0</v>
-      </c>
-      <c r="I15" s="2">
-        <v>0</v>
-      </c>
-      <c r="J15" s="2" t="s">
+      <c r="L31" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>457</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="F32" s="2">
+        <v>0</v>
+      </c>
+      <c r="G32" s="2">
+        <v>0</v>
+      </c>
+      <c r="H32" s="2">
+        <v>0</v>
+      </c>
+      <c r="I32" s="2">
+        <v>0</v>
+      </c>
+      <c r="J32" s="2">
+        <v>0</v>
+      </c>
+      <c r="K32" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
-        <v>479</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>480</v>
-      </c>
-      <c r="E16" s="2">
-        <v>0</v>
-      </c>
-      <c r="F16" s="2">
-        <v>0</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0</v>
-      </c>
-      <c r="H16" s="2">
-        <v>0</v>
-      </c>
-      <c r="I16" s="2">
-        <v>0</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>481</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="E17" s="2">
-        <v>0</v>
-      </c>
-      <c r="F17" s="2">
-        <v>0</v>
-      </c>
-      <c r="G17" s="2">
-        <v>0</v>
-      </c>
-      <c r="H17" s="2">
-        <v>0</v>
-      </c>
-      <c r="I17" s="2">
-        <v>0</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2" t="s">
-        <v>483</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="E18" s="2">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2">
-        <v>0</v>
-      </c>
-      <c r="I18" s="2">
-        <v>0</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>486</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0</v>
-      </c>
-      <c r="F19" s="2">
-        <v>0</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0</v>
-      </c>
-      <c r="H19" s="2">
-        <v>0</v>
-      </c>
-      <c r="I19" s="2">
-        <v>0</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="E20" s="2">
-        <v>0</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>490</v>
-      </c>
-      <c r="E21" s="2">
-        <v>0</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
-      </c>
-      <c r="H21" s="2">
-        <v>0</v>
-      </c>
-      <c r="I21" s="2">
-        <v>0</v>
-      </c>
-      <c r="J21" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K21" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>491</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="E22" s="2">
-        <v>0</v>
-      </c>
-      <c r="F22" s="2">
-        <v>0</v>
-      </c>
-      <c r="G22" s="2">
-        <v>0</v>
-      </c>
-      <c r="H22" s="2">
-        <v>0</v>
-      </c>
-      <c r="I22" s="2">
-        <v>0</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K22" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>494</v>
-      </c>
-      <c r="E23" s="2">
-        <v>0</v>
-      </c>
-      <c r="F23" s="2">
-        <v>0</v>
-      </c>
-      <c r="G23" s="2">
-        <v>0</v>
-      </c>
-      <c r="H23" s="2">
-        <v>0</v>
-      </c>
-      <c r="I23" s="2">
-        <v>0</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>496</v>
-      </c>
-      <c r="E24" s="2">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="E25" s="2">
-        <v>0</v>
-      </c>
-      <c r="F25" s="2">
-        <v>0</v>
-      </c>
-      <c r="G25" s="2">
-        <v>0</v>
-      </c>
-      <c r="H25" s="2">
-        <v>0</v>
-      </c>
-      <c r="I25" s="2">
-        <v>0</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>500</v>
-      </c>
-      <c r="E26" s="2">
-        <v>0</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>501</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="E27" s="2">
-        <v>0</v>
-      </c>
-      <c r="F27" s="2">
-        <v>0</v>
-      </c>
-      <c r="G27" s="2">
-        <v>0</v>
-      </c>
-      <c r="H27" s="2">
-        <v>0</v>
-      </c>
-      <c r="I27" s="2">
-        <v>0</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>452</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="E28" s="2">
-        <v>0</v>
-      </c>
-      <c r="F28" s="2">
-        <v>0</v>
-      </c>
-      <c r="G28" s="2">
-        <v>0</v>
-      </c>
-      <c r="H28" s="2">
-        <v>0</v>
-      </c>
-      <c r="I28" s="2">
-        <v>0</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>506</v>
-      </c>
-      <c r="E29" s="2">
-        <v>0</v>
-      </c>
-      <c r="F29" s="2">
-        <v>0</v>
-      </c>
-      <c r="G29" s="2">
-        <v>0</v>
-      </c>
-      <c r="H29" s="2">
-        <v>0</v>
-      </c>
-      <c r="I29" s="2">
-        <v>0</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="E30" s="2">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2">
-        <v>0</v>
-      </c>
-      <c r="H30" s="2">
-        <v>0</v>
-      </c>
-      <c r="I30" s="2">
-        <v>0</v>
-      </c>
-      <c r="J30" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>509</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>510</v>
-      </c>
-      <c r="E31" s="2">
-        <v>0</v>
-      </c>
-      <c r="F31" s="2">
-        <v>0</v>
-      </c>
-      <c r="G31" s="2">
-        <v>0</v>
-      </c>
-      <c r="H31" s="2">
-        <v>0</v>
-      </c>
-      <c r="I31" s="2">
-        <v>0</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="E32" s="2">
-        <v>0</v>
-      </c>
-      <c r="F32" s="2">
-        <v>0</v>
-      </c>
-      <c r="G32" s="2">
-        <v>0</v>
-      </c>
-      <c r="H32" s="2">
-        <v>0</v>
-      </c>
-      <c r="I32" s="2">
-        <v>0</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="K32" s="2" t="s">
+      <c r="L32" s="2" t="s">
         <v>405</v>
       </c>
     </row>
@@ -3696,19 +3798,19 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>314</v>
@@ -3717,19 +3819,19 @@
         <v>51</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>386</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>393</v>
@@ -3746,7 +3848,7 @@
         <v>55</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>326</v>
@@ -3761,10 +3863,10 @@
         <v>337</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>389</v>
@@ -3787,7 +3889,7 @@
         <v>55</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>340</v>
@@ -3802,10 +3904,10 @@
         <v>337</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>389</v>
@@ -3828,7 +3930,7 @@
         <v>59</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>346</v>
@@ -3843,10 +3945,10 @@
         <v>337</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>389</v>
@@ -3869,7 +3971,7 @@
         <v>63</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>354</v>
@@ -3884,10 +3986,10 @@
         <v>337</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>389</v>
@@ -3910,7 +4012,7 @@
         <v>65</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>362</v>
@@ -3925,10 +4027,10 @@
         <v>337</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>389</v>
@@ -3951,7 +4053,7 @@
         <v>67</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>370</v>
@@ -3966,10 +4068,10 @@
         <v>337</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>389</v>
@@ -3992,7 +4094,7 @@
         <v>69</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>377</v>
@@ -4007,10 +4109,10 @@
         <v>337</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>389</v>
@@ -4024,7 +4126,7 @@
     </row>
     <row r="9" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>157</v>
@@ -4033,7 +4135,7 @@
         <v>158</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>383</v>
@@ -4048,10 +4150,10 @@
         <v>337</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>389</v>
@@ -4083,36 +4185,36 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -4135,7 +4237,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>314</v>
@@ -4144,180 +4246,180 @@
         <v>407</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
     </row>
   </sheetData>
@@ -4340,186 +4442,186 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>339</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
     </row>
   </sheetData>
@@ -7454,7 +7556,7 @@
         <v>389</v>
       </c>
       <c r="E2" s="2">
-        <v>1148</v>
+        <v>1054</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -7490,7 +7592,7 @@
         <v>389</v>
       </c>
       <c r="E4" s="2">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -7508,7 +7610,7 @@
         <v>389</v>
       </c>
       <c r="E5" s="2">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -7526,7 +7628,7 @@
         <v>389</v>
       </c>
       <c r="E6" s="2">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -7544,7 +7646,7 @@
         <v>389</v>
       </c>
       <c r="E7" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -7580,7 +7682,7 @@
         <v>389</v>
       </c>
       <c r="E9" s="2">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F9" s="2"/>
     </row>

</xml_diff>

<commit_message>
Enhanced requirement takes the story from its new @rule tag: the Paris 14-night rule traces to AQPI-34, so the fixed AQPI-4 shows verified in release 2.0
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-e2e-CYC-3/09-report/CYC-3-cycle-report.xlsx
@@ -170,7 +170,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) at 2026-10-02T20:26:12.623Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (452df41) at 2026-10-02T20:28:54.959Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -1704,7 +1704,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T20:26:13.414Z</t>
+    <t>2026-10-02T20:28:55.725Z</t>
   </si>
   <si>
     <t>128 requirements approved; 0 excluded; 0 conflict(s) resolved</t>
@@ -7556,7 +7556,7 @@
         <v>389</v>
       </c>
       <c r="E2" s="2">
-        <v>1054</v>
+        <v>1078</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -7574,7 +7574,7 @@
         <v>389</v>
       </c>
       <c r="E3" s="2">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -7592,7 +7592,7 @@
         <v>389</v>
       </c>
       <c r="E4" s="2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -7610,7 +7610,7 @@
         <v>389</v>
       </c>
       <c r="E5" s="2">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -7628,7 +7628,7 @@
         <v>389</v>
       </c>
       <c r="E6" s="2">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2"/>
     </row>
@@ -7646,7 +7646,7 @@
         <v>389</v>
       </c>
       <c r="E7" s="2">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="F7" s="2"/>
     </row>
@@ -7664,7 +7664,7 @@
         <v>389</v>
       </c>
       <c r="E8" s="2">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -7682,7 +7682,7 @@
         <v>389</v>
       </c>
       <c r="E9" s="2">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="F9" s="2"/>
     </row>

</xml_diff>